<commit_message>
Corrige metodología y artefactos según observaciones de la profesora
</commit_message>
<xml_diff>
--- a/FASE-1/EVIDENCIAS-GRUPALES/Carta Gantt.xlsx
+++ b/FASE-1/EVIDENCIAS-GRUPALES/Carta Gantt.xlsx
@@ -85,7 +85,7 @@
     <t>Requerimientos (iterativo semanal)</t>
   </si>
   <si>
-    <t>Equipo</t>
+    <t>Ezequiel, Lucas, Caro</t>
   </si>
   <si>
     <t>X</t>
@@ -100,7 +100,7 @@
     <t>Hito 1 - Módulo Gestión de Inventario</t>
   </si>
   <si>
-    <t>Ezequiel Suárez</t>
+    <t>Ezequiel, Lucas</t>
   </si>
   <si>
     <t>Hito 2 - Módulo Analítica</t>
@@ -117,7 +117,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00\ [$€-1]"/>
     <numFmt numFmtId="165" formatCode="dd-mm-yyyy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -125,18 +125,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12.0"/>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <b/>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
@@ -181,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -197,28 +192,31 @@
     <xf borderId="1" fillId="2" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -440,7 +438,7 @@
   <cols>
     <col customWidth="1" min="1" max="2" width="8.25"/>
     <col customWidth="1" min="3" max="3" width="32.75"/>
-    <col customWidth="1" min="4" max="4" width="16.13"/>
+    <col customWidth="1" min="4" max="4" width="23.13"/>
     <col customWidth="1" min="5" max="6" width="13.25"/>
     <col customWidth="1" min="7" max="24" width="6.75"/>
     <col customWidth="1" min="25" max="26" width="8.25"/>
@@ -556,67 +554,67 @@
       <c r="C3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="8">
         <v>46237.0</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="8">
         <v>46362.0</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="J3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="K3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="L3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="M3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="N3" s="8" t="s">
+      <c r="N3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="O3" s="8" t="s">
+      <c r="O3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="P3" s="8" t="s">
+      <c r="P3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="Q3" s="8" t="s">
+      <c r="Q3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="R3" s="8" t="s">
+      <c r="R3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="S3" s="8" t="s">
+      <c r="S3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="T3" s="8" t="s">
+      <c r="T3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="U3" s="8" t="s">
+      <c r="U3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="V3" s="8" t="s">
+      <c r="V3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="W3" s="8" t="s">
+      <c r="W3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="X3" s="8" t="s">
+      <c r="X3" s="9" t="s">
         <v>25</v>
       </c>
       <c r="Y3" s="1"/>
@@ -630,67 +628,67 @@
       <c r="C4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="8">
         <v>46237.0</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="8">
         <v>46362.0</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="8" t="s">
+      <c r="H4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="8" t="s">
+      <c r="J4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="K4" s="8" t="s">
+      <c r="K4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="L4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="M4" s="8" t="s">
+      <c r="M4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="N4" s="8" t="s">
+      <c r="N4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="O4" s="8" t="s">
+      <c r="O4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="P4" s="8" t="s">
+      <c r="P4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="Q4" s="8" t="s">
+      <c r="Q4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="R4" s="8" t="s">
+      <c r="R4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="S4" s="8" t="s">
+      <c r="S4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="T4" s="8" t="s">
+      <c r="T4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="U4" s="8" t="s">
+      <c r="U4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="V4" s="8" t="s">
+      <c r="V4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="W4" s="8" t="s">
+      <c r="W4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="X4" s="8" t="s">
+      <c r="X4" s="9" t="s">
         <v>25</v>
       </c>
       <c r="Y4" s="1"/>
@@ -704,67 +702,67 @@
       <c r="C5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="8">
         <v>46237.0</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="8">
         <v>46362.0</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="8" t="s">
+      <c r="I5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="J5" s="8" t="s">
+      <c r="J5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="K5" s="8" t="s">
+      <c r="K5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="L5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="M5" s="8" t="s">
+      <c r="M5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="N5" s="8" t="s">
+      <c r="N5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="O5" s="8" t="s">
+      <c r="O5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="P5" s="8" t="s">
+      <c r="P5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="Q5" s="8" t="s">
+      <c r="Q5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="R5" s="8" t="s">
+      <c r="R5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="S5" s="8" t="s">
+      <c r="S5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="T5" s="8" t="s">
+      <c r="T5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="U5" s="8" t="s">
+      <c r="U5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="V5" s="8" t="s">
+      <c r="V5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="W5" s="8" t="s">
+      <c r="W5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="X5" s="8" t="s">
+      <c r="X5" s="9" t="s">
         <v>25</v>
       </c>
       <c r="Y5" s="1"/>
@@ -778,55 +776,55 @@
       <c r="C6" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="8">
         <v>46237.0</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="8">
         <v>46313.0</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="8" t="s">
+      <c r="I6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="J6" s="8" t="s">
+      <c r="J6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="K6" s="8" t="s">
+      <c r="K6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="L6" s="8" t="s">
+      <c r="L6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="8" t="s">
+      <c r="M6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="N6" s="8" t="s">
+      <c r="N6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="O6" s="8" t="s">
+      <c r="O6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="P6" s="8" t="s">
+      <c r="P6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="Q6" s="8" t="s">
+      <c r="Q6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="R6" s="9"/>
-      <c r="S6" s="9"/>
-      <c r="T6" s="9"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
-      <c r="W6" s="9"/>
-      <c r="X6" s="9"/>
+      <c r="R6" s="10"/>
+      <c r="S6" s="10"/>
+      <c r="T6" s="10"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10"/>
+      <c r="W6" s="10"/>
+      <c r="X6" s="10"/>
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
     </row>
@@ -838,47 +836,47 @@
       <c r="C7" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="8">
         <v>46293.0</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="8">
         <v>46341.0</v>
       </c>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="8" t="s">
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="P7" s="8" t="s">
+      <c r="P7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="Q7" s="8" t="s">
+      <c r="Q7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="R7" s="8" t="s">
+      <c r="R7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="S7" s="8" t="s">
+      <c r="S7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="T7" s="8" t="s">
+      <c r="T7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="U7" s="8" t="s">
+      <c r="U7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="V7" s="8"/>
-      <c r="W7" s="8"/>
-      <c r="X7" s="8"/>
+      <c r="V7" s="9"/>
+      <c r="W7" s="9"/>
+      <c r="X7" s="9"/>
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
     </row>
@@ -887,44 +885,44 @@
       <c r="B8" s="5">
         <v>6.0</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="12">
         <v>46356.0</v>
       </c>
-      <c r="F8" s="11">
+      <c r="F8" s="12">
         <v>46362.0</v>
       </c>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="8"/>
-      <c r="S8" s="8"/>
-      <c r="T8" s="8"/>
-      <c r="U8" s="8"/>
-      <c r="V8" s="8" t="s">
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="9"/>
+      <c r="T8" s="9"/>
+      <c r="U8" s="9"/>
+      <c r="V8" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="W8" s="8" t="s">
+      <c r="W8" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="X8" s="8" t="s">
+      <c r="X8" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="Y8" s="12"/>
-      <c r="Z8" s="12"/>
+      <c r="Y8" s="13"/>
+      <c r="Z8" s="13"/>
     </row>
     <row r="9" ht="17.25" customHeight="1">
       <c r="A9" s="1"/>
@@ -28171,6 +28169,11 @@
       <c r="Z981" s="1"/>
     </row>
   </sheetData>
+  <dataValidations>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D3:D8">
+      <formula1>"Ezequiel,Lucas,Caro"</formula1>
+    </dataValidation>
+  </dataValidations>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>